<commit_message>
data: add OGJ2014 provenance IDs to Excel workbooks
</commit_message>
<xml_diff>
--- a/src/notebooks/ml_data/OGJ2014_extracted_vs_Table1.xlsx
+++ b/src/notebooks/ml_data/OGJ2014_extracted_vs_Table1.xlsx
@@ -42395,7 +42395,7 @@
       </c>
       <c r="U395" t="inlineStr">
         <is>
-          <t>FIELD-0d03f35da104</t>
+          <t>FIELD-35131586bef1</t>
         </is>
       </c>
       <c r="V395" t="inlineStr">
@@ -42426,7 +42426,7 @@
       </c>
       <c r="AB395" t="inlineStr">
         <is>
-          <t>No explicit publication citation/title is present; publication identity was not invented. No source_report column exists; source_report_group_id was not derived from raw_line. Field candidate 'Swan Hills' assigned using a manually reviewed raw_line rule: Swan Hills is the explicit field name; LS is a following lithology abbreviation. case_id is a deterministic hash of exact normalized raw_line; exact repeats share a group.</t>
+          <t>No explicit publication citation/title is present; publication identity was not invented. No source_report column exists; source_report_group_id was not derived from raw_line. Field candidate 'Swan Hills' assigned using a manually reviewed raw_line rule: Swan Hills is the explicit field name; LS is a following lithology abbreviation. Assigned Alberta (Alta.) from corroborating source rows that name the same Swan Hills field; LS is the following lithology abbreviation. case_id is a deterministic hash of exact normalized raw_line; exact repeats share a group.</t>
         </is>
       </c>
       <c r="AC395" t="inlineStr">
@@ -47029,7 +47029,7 @@
       </c>
       <c r="U439" t="inlineStr">
         <is>
-          <t>FIELD-0d03f35da104</t>
+          <t>FIELD-35131586bef1</t>
         </is>
       </c>
       <c r="V439" t="inlineStr">
@@ -47060,7 +47060,7 @@
       </c>
       <c r="AB439" t="inlineStr">
         <is>
-          <t>No explicit publication citation/title is present; publication identity was not invented. No source_report column exists; source_report_group_id was not derived from raw_line. Field candidate 'Swan Hills' assigned using a manually reviewed raw_line rule: Swan Hills is the explicit field name; LS is a following lithology abbreviation. case_id is a deterministic hash of exact normalized raw_line; exact repeats share a group.</t>
+          <t>No explicit publication citation/title is present; publication identity was not invented. No source_report column exists; source_report_group_id was not derived from raw_line. Field candidate 'Swan Hills' assigned using a manually reviewed raw_line rule: Swan Hills is the explicit field name; LS is a following lithology abbreviation. Assigned Alberta (Alta.) from corroborating source rows that name the same Swan Hills field; LS is the following lithology abbreviation. case_id is a deterministic hash of exact normalized raw_line; exact repeats share a group.</t>
         </is>
       </c>
       <c r="AC439" t="inlineStr">
@@ -59615,12 +59615,12 @@
       </c>
       <c r="U559" t="inlineStr">
         <is>
-          <t>FIELD-27c6b7b14062</t>
+          <t>FIELD-7a704168430c</t>
         </is>
       </c>
       <c r="V559" t="inlineStr">
         <is>
-          <t>Arecuna (F.O)</t>
+          <t>Arecuna (F.O.)</t>
         </is>
       </c>
       <c r="W559" t="inlineStr">
@@ -59646,7 +59646,7 @@
       </c>
       <c r="AB559" t="inlineStr">
         <is>
-          <t>No explicit publication citation/title is present; publication identity was not invented. No source_report column exists; source_report_group_id was not derived from raw_line. Field candidate 'Arecuna (F.O)' extracted by the conservative organization/date parser; identity remains provisional. case_id is a deterministic hash of exact normalized raw_line; exact repeats share a group.</t>
+          <t>No explicit publication citation/title is present; publication identity was not invented. No source_report column exists; source_report_group_id was not derived from raw_line. Field candidate 'Arecuna (F.O.)' extracted by the conservative organization/date parser; identity remains provisional. case_id is a deterministic hash of exact normalized raw_line; exact repeats share a group.</t>
         </is>
       </c>
       <c r="AC559" t="inlineStr">
@@ -63932,12 +63932,12 @@
       </c>
       <c r="U600" t="inlineStr">
         <is>
-          <t>FIELD-27c6b7b14062</t>
+          <t>FIELD-7a704168430c</t>
         </is>
       </c>
       <c r="V600" t="inlineStr">
         <is>
-          <t>Arecuna (F.O)</t>
+          <t>Arecuna (F.O.)</t>
         </is>
       </c>
       <c r="W600" t="inlineStr">
@@ -63963,7 +63963,7 @@
       </c>
       <c r="AB600" t="inlineStr">
         <is>
-          <t>No explicit publication citation/title is present; publication identity was not invented. No source_report column exists; source_report_group_id was not derived from raw_line. Field candidate 'Arecuna (F.O)' extracted by the conservative organization/date parser; identity remains provisional. case_id is a deterministic hash of exact normalized raw_line; exact repeats share a group.</t>
+          <t>No explicit publication citation/title is present; publication identity was not invented. No source_report column exists; source_report_group_id was not derived from raw_line. Field candidate 'Arecuna (F.O.)' extracted by the conservative organization/date parser; identity remains provisional. case_id is a deterministic hash of exact normalized raw_line; exact repeats share a group.</t>
         </is>
       </c>
       <c r="AC600" t="inlineStr">

</xml_diff>